<commit_message>
streamlined observation utility to only cover LUCAS relevant entries
</commit_message>
<xml_diff>
--- a/lucas/import_data/utility/observation/excel/preparation.xlsx
+++ b/lucas/import_data/utility/observation/excel/preparation.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="125">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -29,6 +29,9 @@
   </si>
   <si>
     <t xml:space="preserve">display_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">method_pipeline</t>
   </si>
   <si>
     <t xml:space="preserve">abstract</t>
@@ -499,37 +502,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -602,13 +605,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.21"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -624,537 +628,540 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>9</v>
+      <c r="E3" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>12</v>
+      <c r="E4" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>15</v>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
+      <c r="E6" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
+      <c r="E7" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>24</v>
+      <c r="E8" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>27</v>
+      <c r="E9" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="1" t="s">
         <v>31</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="1" t="s">
         <v>35</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="1" t="s">
         <v>39</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="1" t="s">
         <v>43</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="1" t="s">
         <v>47</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" s="1" t="s">
         <v>51</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>54</v>
+      <c r="E16" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>57</v>
+      <c r="E17" s="1" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>60</v>
+      <c r="E18" s="1" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>63</v>
+      <c r="E19" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>66</v>
+      <c r="E20" s="1" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>69</v>
+      <c r="E21" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>72</v>
+      <c r="E22" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>75</v>
+      <c r="E23" s="1" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>78</v>
+      <c r="E24" s="1" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>81</v>
+      <c r="E25" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>84</v>
+      <c r="E26" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>87</v>
+      <c r="E27" s="1" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>90</v>
+      <c r="E28" s="1" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>93</v>
+      <c r="E29" s="1" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>96</v>
+      <c r="E30" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>99</v>
+      <c r="E31" s="1" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>102</v>
+      <c r="E32" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>105</v>
+      <c r="E33" s="1" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>108</v>
+      <c r="E34" s="1" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>111</v>
+      <c r="E35" s="1" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>114</v>
+      <c r="E36" s="1" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>117</v>
+      <c r="E37" s="1" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>120</v>
+      <c r="E38" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>123</v>
+      <c r="E39" s="1" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1162,8 +1169,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>